<commit_message>
Path 1 ENDED (finally) starting path 2 implementation
</commit_message>
<xml_diff>
--- a/public/data/raw/MASTER_RESEARCH.xlsx
+++ b/public/data/raw/MASTER_RESEARCH.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\W12-OPERATOR\Desktop\arcus-platform\public\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BFB9DC3-B3BC-4327-823C-4B0A5C2C3FF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94A1CE06-E453-40C2-9FD1-89E06D2F2733}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{FCFE4B80-8F94-4FB5-A8CE-C44599418DC6}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{FCFE4B80-8F94-4FB5-A8CE-C44599418DC6}"/>
   </bookViews>
   <sheets>
     <sheet name="EVENTS" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10153" uniqueCount="3355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10153" uniqueCount="3356">
   <si>
     <t>B00.01.01</t>
   </si>
@@ -10105,6 +10105,9 @@
   </si>
   <si>
     <t>Corte Brugnatella</t>
+  </si>
+  <si>
+    <t>Asti</t>
   </si>
 </sst>
 </file>
@@ -10571,9 +10574,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema di Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -10611,7 +10614,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -10717,7 +10720,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -10859,7 +10862,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -13908,7 +13911,7 @@
         <v>100</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>19</v>
+        <v>103</v>
       </c>
       <c r="F42" s="6" t="s">
         <v>12</v>
@@ -16039,7 +16042,7 @@
         <v>207</v>
       </c>
       <c r="E71" s="6" t="s">
-        <v>19</v>
+        <v>3355</v>
       </c>
       <c r="F71" s="6" t="s">
         <v>12</v>

</xml_diff>